<commit_message>
Second commit — Interview Automation
</commit_message>
<xml_diff>
--- a/static/excel_practical_template.xlsx
+++ b/static/excel_practical_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView showHorizontalScroll="0" windowWidth="28800" windowHeight="12300" firstSheet="1" activeTab="1"/>
+    <workbookView showHorizontalScroll="0" windowWidth="28800" windowHeight="12300" firstSheet="1" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet5" sheetId="7" state="hidden" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="309">
   <si>
     <t>Name</t>
   </si>
@@ -583,13 +583,208 @@
     <t>Name &amp; Parish</t>
   </si>
   <si>
-    <t>Stbotolph Aldersgate</t>
-  </si>
-  <si>
-    <t>Stclementdanes</t>
-  </si>
-  <si>
-    <t>Stdunstan In The West</t>
+    <t xml:space="preserve"> &amp; Sutton, Surrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Great St Helen, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Andrew Holborn</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Wapping, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Horne, Surrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Hornsoy, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Godmersham, Kent</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Heath, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Aldermanbury, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Martin In The Fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Eastwood, Essex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Bradwell Jaxta Mare, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Ham Charleton Kings, Gloucester</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stbotolph Aldersgate</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Lawrence, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Lomster Horeford</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Martin In The Fields, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Keire Worcester</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Giles In The Fields, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Clement Danes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Blackdon Devon</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Anne Westminster</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St George Botolph Lane, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Boddington, Surrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stoake Northampton</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Sepulchre, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Ampthill, Beds</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Lambeth, Surrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Sepulchre</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Swithin, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stafford</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stclementdanes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Chelsea, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Boreham, Essex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Gadsden, Herts</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stenning Sussex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Dunstan In The West</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Feversham Said County</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Windsor Berks</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stdunstan In The West</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Stanton, Wilts</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; East Grimstead Sussex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Canterbury</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Deale</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Bride, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Edmundthe King Lombard Street, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Giles Cripplegate</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Westminster</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Finchamstead Berks</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Alford Lincoln</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Waltham Abbey, Essex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Islington, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Peter Le Poor</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St James Clerkenwell</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Charlwood, Surrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Rusper Sussex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Sittingbourne, Kent</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Alban Wood Street, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Ickingham, Middlesex</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Mary Whitechapel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Maiden Lane, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Catherine Coleman, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Islington</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; St Botolph Billingsgate</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Nicholas Lane, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Corby Kesteven Lincoln, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Henley On Thames</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &amp; Croydon, Surrey</t>
   </si>
   <si>
     <t>Calculate the Sum, Average, Maximum, and Minimum values of column A in cells B3, C3, D3, and E3 respectively.</t>
@@ -637,7 +832,7 @@
     <t>28</t>
   </si>
   <si>
-    <t>Trim the text in column A, place the trimmed results in column B, and calculate their lengths in column C.</t>
+    <t>Trim the text in column A, place the trimmed results in column B, and calculate Column B lengths in column C.</t>
   </si>
   <si>
     <t>Trim</t>
@@ -2550,15 +2745,15 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>241</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" ht="15" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>184</v>
+        <v>249</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>242</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" ht="15" spans="1:2">
@@ -2988,7 +3183,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>243</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" ht="15" spans="1:1">
@@ -4917,9 +5112,9 @@
   <dimension ref="A1:C81"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="12.1428571428571" style="6" customWidth="1"/>
-    <col min="2" max="2" width="41.7142857142857" style="6" customWidth="1"/>
-    <col min="3" max="3" width="22.7142857142857" style="6" customWidth="1"/>
+    <col min="1" max="1" width="46.5714285714286" style="6" customWidth="1"/>
+    <col min="2" max="2" width="45.7142857142857" style="6" customWidth="1"/>
+    <col min="3" max="3" width="15.2857142857143" style="6" customWidth="1"/>
     <col min="4" max="16384" width="9.14285714285714" style="6"/>
   </cols>
   <sheetData>
@@ -4944,7 +5139,7 @@
         <v>94</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>25</v>
+        <v>180</v>
       </c>
       <c r="C3" s="3"/>
     </row>
@@ -4953,7 +5148,7 @@
         <v>95</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>181</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -4962,7 +5157,7 @@
         <v>96</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>182</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -4971,7 +5166,7 @@
         <v>97</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>28</v>
+        <v>183</v>
       </c>
       <c r="C6" s="3"/>
     </row>
@@ -4980,7 +5175,7 @@
         <v>98</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>29</v>
+        <v>184</v>
       </c>
       <c r="C7" s="3"/>
     </row>
@@ -4989,7 +5184,7 @@
         <v>99</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>30</v>
+        <v>185</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -4998,7 +5193,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>186</v>
       </c>
       <c r="C9" s="3"/>
     </row>
@@ -5007,7 +5202,7 @@
         <v>100</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>32</v>
+        <v>187</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -5016,7 +5211,7 @@
         <v>101</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>33</v>
+        <v>188</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -5025,7 +5220,7 @@
         <v>13</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>34</v>
+        <v>189</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -5034,7 +5229,7 @@
         <v>102</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>35</v>
+        <v>190</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -5043,7 +5238,7 @@
         <v>103</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>36</v>
+        <v>191</v>
       </c>
       <c r="C14" s="3"/>
     </row>
@@ -5052,7 +5247,7 @@
         <v>104</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>37</v>
+        <v>192</v>
       </c>
       <c r="C15" s="3"/>
     </row>
@@ -5061,7 +5256,7 @@
         <v>105</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="C16" s="3"/>
     </row>
@@ -5070,7 +5265,7 @@
         <v>106</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>39</v>
+        <v>194</v>
       </c>
       <c r="C17" s="3"/>
     </row>
@@ -5079,7 +5274,7 @@
         <v>107</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="C18" s="3"/>
     </row>
@@ -5088,7 +5283,7 @@
         <v>108</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>41</v>
+        <v>196</v>
       </c>
       <c r="C19" s="3"/>
     </row>
@@ -5097,7 +5292,7 @@
         <v>109</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>42</v>
+        <v>197</v>
       </c>
       <c r="C20" s="3"/>
     </row>
@@ -5106,7 +5301,7 @@
         <v>110</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>43</v>
+        <v>198</v>
       </c>
       <c r="C21" s="3"/>
     </row>
@@ -5115,7 +5310,7 @@
         <v>111</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>34</v>
+        <v>189</v>
       </c>
       <c r="C22" s="3"/>
     </row>
@@ -5124,7 +5319,7 @@
         <v>112</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>44</v>
+        <v>199</v>
       </c>
       <c r="C23" s="3"/>
     </row>
@@ -5133,7 +5328,7 @@
         <v>113</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>45</v>
+        <v>200</v>
       </c>
       <c r="C24" s="3"/>
     </row>
@@ -5142,7 +5337,7 @@
         <v>18</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>46</v>
+        <v>201</v>
       </c>
       <c r="C25" s="3"/>
     </row>
@@ -5151,7 +5346,7 @@
         <v>114</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>47</v>
+        <v>202</v>
       </c>
       <c r="C26" s="3"/>
     </row>
@@ -5160,7 +5355,7 @@
         <v>115</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>48</v>
+        <v>203</v>
       </c>
       <c r="C27" s="3"/>
     </row>
@@ -5169,7 +5364,7 @@
         <v>12</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>49</v>
+        <v>204</v>
       </c>
       <c r="C28" s="3"/>
     </row>
@@ -5178,7 +5373,7 @@
         <v>116</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>50</v>
+        <v>205</v>
       </c>
       <c r="C29" s="3"/>
     </row>
@@ -5187,7 +5382,7 @@
         <v>117</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>51</v>
+        <v>206</v>
       </c>
       <c r="C30" s="3"/>
     </row>
@@ -5196,7 +5391,7 @@
         <v>118</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>52</v>
+        <v>207</v>
       </c>
       <c r="C31" s="3"/>
     </row>
@@ -5205,7 +5400,7 @@
         <v>14</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>53</v>
+        <v>208</v>
       </c>
       <c r="C32" s="3"/>
     </row>
@@ -5214,7 +5409,7 @@
         <v>119</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>54</v>
+        <v>209</v>
       </c>
       <c r="C33" s="3"/>
     </row>
@@ -5223,7 +5418,7 @@
         <v>120</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>55</v>
+        <v>210</v>
       </c>
       <c r="C34" s="3"/>
     </row>
@@ -5232,7 +5427,7 @@
         <v>16</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="C35" s="3"/>
     </row>
@@ -5241,7 +5436,7 @@
         <v>17</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>57</v>
+        <v>212</v>
       </c>
       <c r="C36" s="3"/>
     </row>
@@ -5250,7 +5445,7 @@
         <v>121</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>58</v>
+        <v>213</v>
       </c>
       <c r="C37" s="3"/>
     </row>
@@ -5259,7 +5454,7 @@
         <v>122</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>59</v>
+        <v>214</v>
       </c>
       <c r="C38" s="3"/>
     </row>
@@ -5268,7 +5463,7 @@
         <v>15</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>60</v>
+        <v>215</v>
       </c>
       <c r="C39" s="3"/>
     </row>
@@ -5277,7 +5472,7 @@
         <v>123</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>61</v>
+        <v>216</v>
       </c>
       <c r="C40" s="3"/>
     </row>
@@ -5286,7 +5481,7 @@
         <v>124</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>62</v>
+        <v>217</v>
       </c>
       <c r="C41" s="3"/>
     </row>
@@ -5295,7 +5490,7 @@
         <v>125</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>63</v>
+        <v>218</v>
       </c>
       <c r="C42" s="3"/>
     </row>
@@ -5304,7 +5499,7 @@
         <v>126</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>182</v>
+        <v>219</v>
       </c>
       <c r="C43" s="3"/>
     </row>
@@ -5313,7 +5508,7 @@
         <v>127</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>65</v>
+        <v>220</v>
       </c>
       <c r="C44" s="3"/>
     </row>
@@ -5322,7 +5517,7 @@
         <v>128</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>66</v>
+        <v>221</v>
       </c>
       <c r="C45" s="3"/>
     </row>
@@ -5331,7 +5526,7 @@
         <v>129</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>67</v>
+        <v>222</v>
       </c>
       <c r="C46" s="3"/>
     </row>
@@ -5340,7 +5535,7 @@
         <v>130</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>68</v>
+        <v>223</v>
       </c>
       <c r="C47" s="3"/>
     </row>
@@ -5349,7 +5544,7 @@
         <v>131</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>69</v>
+        <v>224</v>
       </c>
       <c r="C48" s="3"/>
     </row>
@@ -5358,7 +5553,7 @@
         <v>132</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>53</v>
+        <v>208</v>
       </c>
       <c r="C49" s="3"/>
     </row>
@@ -5367,7 +5562,7 @@
         <v>133</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>69</v>
+        <v>224</v>
       </c>
       <c r="C50" s="3"/>
     </row>
@@ -5376,7 +5571,7 @@
         <v>134</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>34</v>
+        <v>189</v>
       </c>
       <c r="C51" s="3"/>
     </row>
@@ -5385,7 +5580,7 @@
         <v>135</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>70</v>
+        <v>225</v>
       </c>
       <c r="C52" s="3"/>
     </row>
@@ -5394,7 +5589,7 @@
         <v>136</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>71</v>
+        <v>226</v>
       </c>
       <c r="C53" s="3"/>
     </row>
@@ -5403,7 +5598,7 @@
         <v>137</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>72</v>
+        <v>227</v>
       </c>
       <c r="C54" s="3"/>
     </row>
@@ -5412,7 +5607,7 @@
         <v>138</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>73</v>
+        <v>228</v>
       </c>
       <c r="C55" s="3"/>
     </row>
@@ -5421,7 +5616,7 @@
         <v>139</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>27</v>
+        <v>182</v>
       </c>
       <c r="C56" s="4"/>
     </row>
@@ -5430,7 +5625,7 @@
         <v>140</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>74</v>
+        <v>229</v>
       </c>
       <c r="C57" s="3"/>
     </row>
@@ -5439,7 +5634,7 @@
         <v>141</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>75</v>
+        <v>230</v>
       </c>
       <c r="C58" s="3"/>
     </row>
@@ -5448,7 +5643,7 @@
         <v>142</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>76</v>
+        <v>231</v>
       </c>
       <c r="C59" s="3"/>
     </row>
@@ -5457,7 +5652,7 @@
         <v>143</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>63</v>
+        <v>218</v>
       </c>
       <c r="C60" s="3"/>
     </row>
@@ -5466,7 +5661,7 @@
         <v>144</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>77</v>
+        <v>232</v>
       </c>
       <c r="C61" s="3"/>
     </row>
@@ -5475,7 +5670,7 @@
         <v>145</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>34</v>
+        <v>189</v>
       </c>
       <c r="C62" s="3"/>
     </row>
@@ -5484,7 +5679,7 @@
         <v>146</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>78</v>
+        <v>233</v>
       </c>
       <c r="C63" s="3"/>
     </row>
@@ -5493,7 +5688,7 @@
         <v>147</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>79</v>
+        <v>234</v>
       </c>
       <c r="C64" s="3"/>
     </row>
@@ -5502,7 +5697,7 @@
         <v>148</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>61</v>
+        <v>216</v>
       </c>
       <c r="C65" s="3"/>
     </row>
@@ -5511,7 +5706,7 @@
         <v>149</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>34</v>
+        <v>189</v>
       </c>
       <c r="C66" s="3"/>
     </row>
@@ -5520,7 +5715,7 @@
         <v>150</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>52</v>
+        <v>207</v>
       </c>
       <c r="C67" s="3"/>
     </row>
@@ -5529,7 +5724,7 @@
         <v>151</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>80</v>
+        <v>235</v>
       </c>
       <c r="C68" s="3"/>
     </row>
@@ -5538,7 +5733,7 @@
         <v>152</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>81</v>
+        <v>236</v>
       </c>
       <c r="C69" s="3"/>
     </row>
@@ -5547,7 +5742,7 @@
         <v>153</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="C70" s="3"/>
     </row>
@@ -5556,7 +5751,7 @@
         <v>154</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>76</v>
+        <v>231</v>
       </c>
       <c r="C71" s="3"/>
     </row>
@@ -5565,7 +5760,7 @@
         <v>8</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>83</v>
+        <v>238</v>
       </c>
       <c r="C72" s="3"/>
     </row>
@@ -5574,7 +5769,7 @@
         <v>11</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>84</v>
+        <v>239</v>
       </c>
       <c r="C73" s="3"/>
     </row>
@@ -5583,7 +5778,7 @@
         <v>155</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>85</v>
+        <v>240</v>
       </c>
       <c r="C74" s="3"/>
     </row>
@@ -5592,7 +5787,7 @@
         <v>156</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>86</v>
+        <v>241</v>
       </c>
       <c r="C75" s="3"/>
     </row>
@@ -5601,7 +5796,7 @@
         <v>5</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>87</v>
+        <v>242</v>
       </c>
       <c r="C76" s="3"/>
     </row>
@@ -5610,7 +5805,7 @@
         <v>157</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>88</v>
+        <v>243</v>
       </c>
       <c r="C77" s="3"/>
     </row>
@@ -5619,7 +5814,7 @@
         <v>158</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>89</v>
+        <v>244</v>
       </c>
       <c r="C78" s="3"/>
     </row>
@@ -5628,7 +5823,7 @@
         <v>159</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>90</v>
+        <v>245</v>
       </c>
       <c r="C79" s="3"/>
     </row>
@@ -5637,7 +5832,7 @@
         <v>160</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>91</v>
+        <v>246</v>
       </c>
       <c r="C80" s="3"/>
     </row>
@@ -5646,7 +5841,7 @@
         <v>161</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>92</v>
+        <v>247</v>
       </c>
       <c r="C81" s="3"/>
     </row>
@@ -5669,24 +5864,24 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" ht="15" spans="1:5">
       <c r="A2" s="8" t="s">
-        <v>184</v>
+        <v>249</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>185</v>
+        <v>250</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>186</v>
+        <v>251</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>187</v>
+        <v>252</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>188</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" ht="15" spans="1:5">
@@ -6421,7 +6616,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -6429,7 +6624,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>190</v>
+        <v>255</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>163</v>
@@ -6443,7 +6638,7 @@
         <v>98</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>191</v>
+        <v>256</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>167</v>
@@ -6457,7 +6652,7 @@
         <v>101</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>192</v>
+        <v>257</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>168</v>
@@ -6471,7 +6666,7 @@
         <v>95</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>193</v>
+        <v>258</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>165</v>
@@ -6485,7 +6680,7 @@
         <v>99</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>194</v>
+        <v>259</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>167</v>
@@ -6499,7 +6694,7 @@
         <v>94</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>194</v>
+        <v>259</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>164</v>
@@ -6513,7 +6708,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>194</v>
+        <v>259</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>167</v>
@@ -6527,7 +6722,7 @@
         <v>100</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>195</v>
+        <v>260</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>167</v>
@@ -6541,7 +6736,7 @@
         <v>96</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>191</v>
+        <v>256</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>165</v>
@@ -6555,7 +6750,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>196</v>
+        <v>261</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>168</v>
@@ -6569,7 +6764,7 @@
         <v>97</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>197</v>
+        <v>262</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>166</v>
@@ -6601,7 +6796,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>198</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -6609,71 +6804,71 @@
         <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>199</v>
+        <v>264</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>200</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="3" t="s">
-        <v>201</v>
+        <v>266</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
-        <v>202</v>
+        <v>267</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="3" t="s">
-        <v>203</v>
+        <v>268</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="3" t="s">
-        <v>204</v>
+        <v>269</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="3" t="s">
-        <v>205</v>
+        <v>270</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="3" t="s">
-        <v>206</v>
+        <v>271</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="3" t="s">
-        <v>207</v>
+        <v>272</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="3" t="s">
-        <v>208</v>
+        <v>273</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="3" t="s">
-        <v>209</v>
+        <v>274</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -6687,21 +6882,21 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="3" t="s">
-        <v>210</v>
+        <v>275</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="3" t="s">
-        <v>211</v>
+        <v>276</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="3" t="s">
-        <v>212</v>
+        <v>277</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -6715,7 +6910,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="3" t="s">
-        <v>213</v>
+        <v>278</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -6729,7 +6924,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="3" t="s">
-        <v>214</v>
+        <v>279</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -6743,7 +6938,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="3" t="s">
-        <v>215</v>
+        <v>280</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -6778,14 +6973,14 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="3" t="s">
-        <v>216</v>
+        <v>281</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="3" t="s">
-        <v>217</v>
+        <v>282</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -6799,21 +6994,21 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="3" t="s">
-        <v>218</v>
+        <v>283</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="3" t="s">
-        <v>219</v>
+        <v>284</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="3" t="s">
-        <v>220</v>
+        <v>285</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -6827,7 +7022,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="3" t="s">
-        <v>221</v>
+        <v>286</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
@@ -6848,21 +7043,21 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="3" t="s">
-        <v>222</v>
+        <v>287</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="3" t="s">
-        <v>223</v>
+        <v>288</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="3" t="s">
-        <v>224</v>
+        <v>289</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -6932,7 +7127,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="3" t="s">
-        <v>225</v>
+        <v>290</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -6946,7 +7141,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="3" t="s">
-        <v>225</v>
+        <v>290</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
@@ -6960,7 +7155,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="3" t="s">
-        <v>226</v>
+        <v>291</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
@@ -7002,14 +7197,14 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="3" t="s">
-        <v>227</v>
+        <v>292</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="3" t="s">
-        <v>228</v>
+        <v>293</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
@@ -7044,7 +7239,7 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="3" t="s">
-        <v>229</v>
+        <v>294</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7"/>
@@ -7065,7 +7260,7 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="3" t="s">
-        <v>220</v>
+        <v>285</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7"/>
@@ -7079,28 +7274,28 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="3" t="s">
-        <v>230</v>
+        <v>295</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7"/>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="3" t="s">
-        <v>231</v>
+        <v>296</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7"/>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="3" t="s">
-        <v>228</v>
+        <v>293</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7"/>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="3" t="s">
-        <v>232</v>
+        <v>297</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7"/>
@@ -7114,14 +7309,14 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" s="3" t="s">
-        <v>233</v>
+        <v>298</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7"/>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" s="3" t="s">
-        <v>234</v>
+        <v>299</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
@@ -7142,14 +7337,14 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="3" t="s">
-        <v>235</v>
+        <v>300</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7"/>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" s="3" t="s">
-        <v>236</v>
+        <v>301</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7"/>
@@ -7163,7 +7358,7 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" s="3" t="s">
-        <v>237</v>
+        <v>302</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7"/>
@@ -7188,7 +7383,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" s="6" customFormat="1" spans="1:3">
@@ -7196,10 +7391,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>239</v>
+        <v>304</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>240</v>
+        <v>305</v>
       </c>
     </row>
     <row r="3" s="6" customFormat="1" spans="1:3">
@@ -7755,30 +7950,40 @@
       <c r="B81" s="7"/>
       <c r="C81" s="7"/>
     </row>
-    <row r="82" spans="1:1">
-      <c r="A82" s="6" t="s">
+    <row r="82" spans="1:3">
+      <c r="A82" s="3" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="83" spans="1:1">
-      <c r="A83" s="6" t="s">
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="84" spans="1:1">
-      <c r="A84" s="6" t="s">
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="3" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="85" spans="1:1">
-      <c r="A85" s="6" t="s">
+      <c r="B84" s="7"/>
+      <c r="C84" s="7"/>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="3" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="86" spans="1:1">
-      <c r="A86" s="6" t="s">
+      <c r="B85" s="7"/>
+      <c r="C85" s="7"/>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" s="3" t="s">
         <v>106</v>
       </c>
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>